<commit_message>
Support per-group cascade start and multi-group dashboard layout
Per-group cascade start:
- New optional "Cascade Start" column on the Tickets tab, set on one row per
  group; falls back to Config ticket_cascade_start so groups can stagger
- TicketItem.cascadeStartISO; computeTicketGroup resolves the per-group start
- sheets.ts parses the column; +1 unit test (19 passing)

Dashboard layout for multiple ticket groups:
- New TicketGroupSummary compact card; the dashboard spotlights the
  soonest-closing group as a full panel and shows the rest as compact cards
- demo data now spans 3 staggered groups to exercise the layout

Also: regenerated import workbook/CSVs with the Cascade Start column, updated
sheet template docs, and refreshed the Session 1 handoff log.

https://claude.ai/code/session_019XgPpYxiBLSsK5yaWdd13H
</commit_message>
<xml_diff>
--- a/docs/Silent-Auction-Import.xlsx
+++ b/docs/Silent-Auction-Import.xlsx
@@ -876,7 +876,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K29"/>
+  <dimension ref="A1:L29"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -884,11 +884,12 @@
     <col min="4" max="4" width="11.83203125" customWidth="1"/>
     <col min="5" max="5" width="11.83203125" customWidth="1"/>
     <col min="6" max="6" width="18.83203125" customWidth="1"/>
-    <col min="7" max="7" width="16.83203125" customWidth="1"/>
-    <col min="8" max="8" width="48.83203125" customWidth="1"/>
-    <col min="9" max="9" width="16.83203125" customWidth="1"/>
-    <col min="10" max="10" width="7.83203125" customWidth="1"/>
-    <col min="11" max="11" width="10.83203125" customWidth="1"/>
+    <col min="7" max="7" width="14.83203125" customWidth="1"/>
+    <col min="8" max="8" width="16.83203125" customWidth="1"/>
+    <col min="9" max="9" width="48.83203125" customWidth="1"/>
+    <col min="10" max="10" width="16.83203125" customWidth="1"/>
+    <col min="11" max="11" width="7.83203125" customWidth="1"/>
+    <col min="12" max="12" width="10.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -911,18 +912,21 @@
         <v>High Bidder</v>
       </c>
       <c r="G1" t="str">
+        <v>Cascade Start</v>
+      </c>
+      <c r="H1" t="str">
         <v>Last Bid Time</v>
       </c>
-      <c r="H1" t="str">
+      <c r="I1" t="str">
         <v>Notes</v>
       </c>
-      <c r="I1" t="str">
+      <c r="J1" t="str">
         <v>Winner Phone</v>
       </c>
-      <c r="J1" t="str">
+      <c r="K1" t="str">
         <v>Paid?</v>
       </c>
-      <c r="K1" t="str">
+      <c r="L1" t="str">
         <v>Picked Up?</v>
       </c>
     </row>
@@ -946,18 +950,21 @@
         <v>Matt Hershberger</v>
       </c>
       <c r="G2" t="str">
-        <v/>
+        <v>7:00 PM</v>
       </c>
       <c r="H2" t="str">
+        <v/>
+      </c>
+      <c r="I2" t="str">
         <v>Lunch on Jul 23</v>
       </c>
-      <c r="I2" t="str">
-        <v/>
-      </c>
       <c r="J2" t="str">
         <v/>
       </c>
       <c r="K2" t="str">
+        <v/>
+      </c>
+      <c r="L2" t="str">
         <v/>
       </c>
     </row>
@@ -984,15 +991,18 @@
         <v/>
       </c>
       <c r="H3" t="str">
+        <v/>
+      </c>
+      <c r="I3" t="str">
         <v>Lunch on Jul 23</v>
       </c>
-      <c r="I3" t="str">
-        <v/>
-      </c>
       <c r="J3" t="str">
         <v/>
       </c>
       <c r="K3" t="str">
+        <v/>
+      </c>
+      <c r="L3" t="str">
         <v/>
       </c>
     </row>
@@ -1019,15 +1029,18 @@
         <v/>
       </c>
       <c r="H4" t="str">
+        <v/>
+      </c>
+      <c r="I4" t="str">
         <v>Lunch on Jul 23</v>
       </c>
-      <c r="I4" t="str">
-        <v/>
-      </c>
       <c r="J4" t="str">
         <v/>
       </c>
       <c r="K4" t="str">
+        <v/>
+      </c>
+      <c r="L4" t="str">
         <v/>
       </c>
     </row>
@@ -1054,15 +1067,18 @@
         <v/>
       </c>
       <c r="H5" t="str">
+        <v/>
+      </c>
+      <c r="I5" t="str">
         <v>Lunch on Jul 23</v>
       </c>
-      <c r="I5" t="str">
-        <v/>
-      </c>
       <c r="J5" t="str">
         <v/>
       </c>
       <c r="K5" t="str">
+        <v/>
+      </c>
+      <c r="L5" t="str">
         <v/>
       </c>
     </row>
@@ -1089,15 +1105,18 @@
         <v/>
       </c>
       <c r="H6" t="str">
+        <v/>
+      </c>
+      <c r="I6" t="str">
         <v>Lunch on Jul 23</v>
       </c>
-      <c r="I6" t="str">
-        <v/>
-      </c>
       <c r="J6" t="str">
         <v/>
       </c>
       <c r="K6" t="str">
+        <v/>
+      </c>
+      <c r="L6" t="str">
         <v/>
       </c>
     </row>
@@ -1124,15 +1143,18 @@
         <v/>
       </c>
       <c r="H7" t="str">
+        <v/>
+      </c>
+      <c r="I7" t="str">
         <v>Lunch on Jul 23</v>
       </c>
-      <c r="I7" t="str">
-        <v/>
-      </c>
       <c r="J7" t="str">
         <v/>
       </c>
       <c r="K7" t="str">
+        <v/>
+      </c>
+      <c r="L7" t="str">
         <v/>
       </c>
     </row>
@@ -1159,15 +1181,18 @@
         <v/>
       </c>
       <c r="H8" t="str">
+        <v/>
+      </c>
+      <c r="I8" t="str">
         <v>Lunch on Jul 23</v>
       </c>
-      <c r="I8" t="str">
-        <v/>
-      </c>
       <c r="J8" t="str">
         <v/>
       </c>
       <c r="K8" t="str">
+        <v/>
+      </c>
+      <c r="L8" t="str">
         <v/>
       </c>
     </row>
@@ -1194,15 +1219,18 @@
         <v/>
       </c>
       <c r="H9" t="str">
+        <v/>
+      </c>
+      <c r="I9" t="str">
         <v>Lunch on Jul 23</v>
       </c>
-      <c r="I9" t="str">
-        <v/>
-      </c>
       <c r="J9" t="str">
         <v/>
       </c>
       <c r="K9" t="str">
+        <v/>
+      </c>
+      <c r="L9" t="str">
         <v/>
       </c>
     </row>
@@ -1229,15 +1257,18 @@
         <v/>
       </c>
       <c r="H10" t="str">
+        <v/>
+      </c>
+      <c r="I10" t="str">
         <v>Lunch on Jul 23</v>
       </c>
-      <c r="I10" t="str">
-        <v/>
-      </c>
       <c r="J10" t="str">
         <v/>
       </c>
       <c r="K10" t="str">
+        <v/>
+      </c>
+      <c r="L10" t="str">
         <v/>
       </c>
     </row>
@@ -1264,15 +1295,18 @@
         <v/>
       </c>
       <c r="H11" t="str">
+        <v/>
+      </c>
+      <c r="I11" t="str">
         <v>Lunch on Jul 23</v>
       </c>
-      <c r="I11" t="str">
-        <v/>
-      </c>
       <c r="J11" t="str">
         <v/>
       </c>
       <c r="K11" t="str">
+        <v/>
+      </c>
+      <c r="L11" t="str">
         <v/>
       </c>
     </row>
@@ -1299,15 +1333,18 @@
         <v/>
       </c>
       <c r="H12" t="str">
+        <v/>
+      </c>
+      <c r="I12" t="str">
         <v>Lunch on Jul 23</v>
       </c>
-      <c r="I12" t="str">
-        <v/>
-      </c>
       <c r="J12" t="str">
         <v/>
       </c>
       <c r="K12" t="str">
+        <v/>
+      </c>
+      <c r="L12" t="str">
         <v/>
       </c>
     </row>
@@ -1334,15 +1371,18 @@
         <v/>
       </c>
       <c r="H13" t="str">
+        <v/>
+      </c>
+      <c r="I13" t="str">
         <v>Lunch on Jul 23</v>
       </c>
-      <c r="I13" t="str">
-        <v/>
-      </c>
       <c r="J13" t="str">
         <v/>
       </c>
       <c r="K13" t="str">
+        <v/>
+      </c>
+      <c r="L13" t="str">
         <v/>
       </c>
     </row>
@@ -1366,18 +1406,21 @@
         <v>Matt Janzi</v>
       </c>
       <c r="G14" t="str">
-        <v/>
+        <v>7:20 PM</v>
       </c>
       <c r="H14" t="str">
+        <v/>
+      </c>
+      <c r="I14" t="str">
         <v>@ Peter's house 7/10 at 5:30. Campfire after, weather permitting</v>
       </c>
-      <c r="I14" t="str">
-        <v/>
-      </c>
       <c r="J14" t="str">
         <v/>
       </c>
       <c r="K14" t="str">
+        <v/>
+      </c>
+      <c r="L14" t="str">
         <v/>
       </c>
     </row>
@@ -1415,6 +1458,9 @@
       <c r="K15" t="str">
         <v/>
       </c>
+      <c r="L15" t="str">
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
@@ -1450,6 +1496,9 @@
       <c r="K16" t="str">
         <v/>
       </c>
+      <c r="L16" t="str">
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
@@ -1485,6 +1534,9 @@
       <c r="K17" t="str">
         <v/>
       </c>
+      <c r="L17" t="str">
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
@@ -1506,18 +1558,21 @@
         <v>Aaron Troyer</v>
       </c>
       <c r="G18" t="str">
-        <v/>
+        <v>7:35 PM</v>
       </c>
       <c r="H18" t="str">
+        <v/>
+      </c>
+      <c r="I18" t="str">
         <v>Donated by Dennis · Sometime in July</v>
       </c>
-      <c r="I18" t="str">
-        <v/>
-      </c>
       <c r="J18" t="str">
         <v/>
       </c>
       <c r="K18" t="str">
+        <v/>
+      </c>
+      <c r="L18" t="str">
         <v/>
       </c>
     </row>
@@ -1544,15 +1599,18 @@
         <v/>
       </c>
       <c r="H19" t="str">
+        <v/>
+      </c>
+      <c r="I19" t="str">
         <v>Donated by Dennis · Sometime in July</v>
       </c>
-      <c r="I19" t="str">
-        <v/>
-      </c>
       <c r="J19" t="str">
         <v/>
       </c>
       <c r="K19" t="str">
+        <v/>
+      </c>
+      <c r="L19" t="str">
         <v/>
       </c>
     </row>
@@ -1579,15 +1637,18 @@
         <v/>
       </c>
       <c r="H20" t="str">
+        <v/>
+      </c>
+      <c r="I20" t="str">
         <v>Donated by Dennis · Sometime in July</v>
       </c>
-      <c r="I20" t="str">
-        <v/>
-      </c>
       <c r="J20" t="str">
         <v/>
       </c>
       <c r="K20" t="str">
+        <v/>
+      </c>
+      <c r="L20" t="str">
         <v/>
       </c>
     </row>
@@ -1611,18 +1672,21 @@
         <v>Dan D. I. Miller</v>
       </c>
       <c r="G21" t="str">
-        <v/>
+        <v>7:45 PM</v>
       </c>
       <c r="H21" t="str">
+        <v/>
+      </c>
+      <c r="I21" t="str">
         <v>Donated by Charles &amp; Gloria Kratzer</v>
       </c>
-      <c r="I21" t="str">
-        <v/>
-      </c>
       <c r="J21" t="str">
         <v/>
       </c>
       <c r="K21" t="str">
+        <v/>
+      </c>
+      <c r="L21" t="str">
         <v/>
       </c>
     </row>
@@ -1649,15 +1713,18 @@
         <v/>
       </c>
       <c r="H22" t="str">
+        <v/>
+      </c>
+      <c r="I22" t="str">
         <v>Donated by Charles &amp; Gloria Kratzer</v>
       </c>
-      <c r="I22" t="str">
-        <v/>
-      </c>
       <c r="J22" t="str">
         <v/>
       </c>
       <c r="K22" t="str">
+        <v/>
+      </c>
+      <c r="L22" t="str">
         <v/>
       </c>
     </row>
@@ -1681,18 +1748,21 @@
         <v>Eric McGlumphy</v>
       </c>
       <c r="G23" t="str">
-        <v/>
+        <v>7:55 PM</v>
       </c>
       <c r="H23" t="str">
+        <v/>
+      </c>
+      <c r="I23" t="str">
         <v>Donated by Albert &amp; Derrick W · 2 people per ticket</v>
       </c>
-      <c r="I23" t="str">
-        <v/>
-      </c>
       <c r="J23" t="str">
         <v/>
       </c>
       <c r="K23" t="str">
+        <v/>
+      </c>
+      <c r="L23" t="str">
         <v/>
       </c>
     </row>
@@ -1719,15 +1789,18 @@
         <v/>
       </c>
       <c r="H24" t="str">
+        <v/>
+      </c>
+      <c r="I24" t="str">
         <v>Donated by Albert &amp; Derrick W · 2 people per ticket</v>
       </c>
-      <c r="I24" t="str">
-        <v/>
-      </c>
       <c r="J24" t="str">
         <v/>
       </c>
       <c r="K24" t="str">
+        <v/>
+      </c>
+      <c r="L24" t="str">
         <v/>
       </c>
     </row>
@@ -1754,15 +1827,18 @@
         <v/>
       </c>
       <c r="H25" t="str">
+        <v/>
+      </c>
+      <c r="I25" t="str">
         <v>Donated by Albert &amp; Derrick W · 2 people per ticket</v>
       </c>
-      <c r="I25" t="str">
-        <v/>
-      </c>
       <c r="J25" t="str">
         <v/>
       </c>
       <c r="K25" t="str">
+        <v/>
+      </c>
+      <c r="L25" t="str">
         <v/>
       </c>
     </row>
@@ -1789,15 +1865,18 @@
         <v/>
       </c>
       <c r="H26" t="str">
+        <v/>
+      </c>
+      <c r="I26" t="str">
         <v>Donated by Albert &amp; Derrick W · 2 people per ticket</v>
       </c>
-      <c r="I26" t="str">
-        <v/>
-      </c>
       <c r="J26" t="str">
         <v/>
       </c>
       <c r="K26" t="str">
+        <v/>
+      </c>
+      <c r="L26" t="str">
         <v/>
       </c>
     </row>
@@ -1824,15 +1903,18 @@
         <v/>
       </c>
       <c r="H27" t="str">
+        <v/>
+      </c>
+      <c r="I27" t="str">
         <v>Donated by Albert &amp; Derrick W · 2 people per ticket</v>
       </c>
-      <c r="I27" t="str">
-        <v/>
-      </c>
       <c r="J27" t="str">
         <v/>
       </c>
       <c r="K27" t="str">
+        <v/>
+      </c>
+      <c r="L27" t="str">
         <v/>
       </c>
     </row>
@@ -1859,15 +1941,18 @@
         <v/>
       </c>
       <c r="H28" t="str">
+        <v/>
+      </c>
+      <c r="I28" t="str">
         <v>Donated by Albert &amp; Derrick W · 2 people per ticket</v>
       </c>
-      <c r="I28" t="str">
-        <v/>
-      </c>
       <c r="J28" t="str">
         <v/>
       </c>
       <c r="K28" t="str">
+        <v/>
+      </c>
+      <c r="L28" t="str">
         <v/>
       </c>
     </row>
@@ -1894,21 +1979,24 @@
         <v/>
       </c>
       <c r="H29" t="str">
+        <v/>
+      </c>
+      <c r="I29" t="str">
         <v>Watching only · all-you-can-eat wings</v>
       </c>
-      <c r="I29" t="str">
-        <v/>
-      </c>
       <c r="J29" t="str">
         <v/>
       </c>
       <c r="K29" t="str">
+        <v/>
+      </c>
+      <c r="L29" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K29"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L29"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>